<commit_message>
x data ingestion complete (missing dates) and still historical data only.
</commit_message>
<xml_diff>
--- a/design_decisions.xlsx
+++ b/design_decisions.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1527,6 +1527,51 @@
       <c r="I23" s="2" t="inlineStr">
         <is>
           <t>src/screen_tickers.py; data/reference/ticker_classification.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Theme scanning: tokenise once + hash lookups</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>The original theme scanner ran ~20 separate keyword regexes over every post's full text. At ~130-600 posts/sec, a one-year window (2.8M posts) meant HOURS per notebook-04 run - too slow to iterate on.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>One pass per post: lowercase the text once, tokenise with a single regex ([a-z0-9]+), then look every token up in a prebuilt dict {word -&gt; themes} (O(1) per token, regardless of how many keywords exist). Multi-word phrases ('short squeeze', 'data center') are checked with Python's C-level substring 'in' against the lowered text. Per-post set semantics kept: a post counts at most once per theme.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Option considered: one combined pre-compiled regex per theme + pandas str.count (vectorised). Hash lookups won: cost is O(tokens in post), not O(number of keywords), so adding keywords is free.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Measured on real data (100k-post benchmark): 12,298 posts/sec -&gt; the full 2.8M-post window takes ~4 minutes instead of ~6 hours (~95x). Stale 'many HOURS' warnings removed from WEEK2.md and notebook 01.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Single-word keywords must match a whole token exactly - plurals/variants need listing explicitly ('chip' AND 'chips'). Phrases are still scanned per post (fast C substring, but linear in phrase count).</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>src/themes.py (themes_in_text, _get_keyword_lookup)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sentiment data from hugging face
- Implemented sentiment scoring for posts using VADER and a custom WSB/finance lexicon in `sentiment.py`.
- Added functions for scoring text, adding sentiment to DataFrames, and aggregating daily sentiment by ticker and theme.
</commit_message>
<xml_diff>
--- a/design_decisions.xlsx
+++ b/design_decisions.xlsx
@@ -92,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -113,6 +113,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -479,18 +482,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -501,40 +505,45 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Date (approx.)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>The decision</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Why a decision was needed (the problem)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>What was decided (technical)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Standard / alternative approach</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Outcome / result</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Trade-off / known cost</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Where it lives</t>
         </is>
@@ -544,42 +553,47 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>One parquet, subreddit-blocked row groups</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Data engineering</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>15 separate .zst dumps (~3 GB of compressed JSON, 7.95M posts). Decompressing and JSON-parsing them for every analysis run took hours - iteration was impossible.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>One-time ETL (prep_posts.py): stream each dump, clean each record, write ONE pyarrow parquet whose row groups are laid out in subreddit blocks. Each row group carries min/max column stats, so filtered reads (subreddit IN [...], date &gt;= ...) are pushed down into the reader and non-matching blocks are skipped entirely.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Keep per-subreddit files, load JSON on demand, or stand up a database (DuckDB/SQLite).</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>1.15 GB single file, 34 row groups. Metadata peek is instant; a one-subreddit read touches ~1/30th of the file; a full 2021 slice (2.8M posts) loads in seconds-to-minutes. Notebooks never touch raw files again.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>If cleaning rules change, the parquet must be rebuilt from the dumps (which is why the dumps are kept as the immutable source of truth).</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>data_ingestion/scripts/prep_posts.py</t>
         </is>
@@ -589,42 +603,47 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Universal 8-column schema</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Data engineering</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Sources have different shapes (torrent dumps, CSV/Kaggle exports, future live PRAW JSON). Analysis code that knows about source-specific fields breaks every time a new source arrives.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>normalise() maps EVERY record to exactly: id, date, author, score, subreddit, title, selftext, num_comments. Dates normalised to 'YYYY-MM-DD' strings, subreddits lowercased. Downstream code is only allowed to know these 8 columns.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Keep each source's native fields and adapt per analysis.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Notebooks 02-05 and all 20 tests run unchanged on any source that maps to the shape. The live-ingestion spec is one sentence: 'normalise to the same 8 columns'.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Potentially useful fields (flair, upvote_ratio, URLs) are discarded at ingestion.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>src/clean_data.py</t>
         </is>
@@ -634,42 +653,47 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Dedup: first seen wins</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Data engineering</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>The archive crawled 4 pinned WSB posts twice (5 extra rows), and future live re-fetches will see already-known post ids again. Without one rule, historical and live data would disagree.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Keep the FIRST occurrence of each post id, drop all later ones - the same deterministic rule for the historical backfill and for planned live appends. The 5 existing duplicate rows were documented and left in place (immaterial) rather than hand-editing a 1.15 GB parquet.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Ad-hoc dedup per load, or 'latest wins' (keeps post edits).</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Deterministic, rebuild-stable dataset. A pytest pins duplicates &lt;= 5 and the count may only ever go DOWN - new duplicates fail the suite loudly.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>'First seen' keeps the earliest snapshot, so later title/body edits are not captured.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>prep_posts.py; tests/test_pipeline.py</t>
         </is>
@@ -679,42 +703,47 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Upvote weighting = score squared</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Signal construction</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Raw counts treat a 50k-upvote viral post and a bot's ignored post identically - the signal is trivially spam-able by posting volume.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>weighted_count = sum(score^2) over posts mentioning the ticker that day, kept ALONGSIDE the unweighted mention_count. Squaring is a deliberate power law: 1,000 upvotes contributes 1,000,000 vs 100 for 10 upvotes - crowd-endorsed posts dominate by design.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Linear score weighting, or log(1+score) dampening (both dampen virality).</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>daily_ticker_counts.parquet carries BOTH series. The raw count acts as the maturity-bias-immune baseline that gets validated first; the weighted one captures virality.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Highly sensitive to score-maturity bias and to one mega-post; softening to score or log(1+score) is the documented fallback if the back-test says so.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>src/build_mentions.py; README 'Weighting assumptions'</t>
         </is>
@@ -724,42 +753,47 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Per-post mention dedup</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Signal construction</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>One verbose poster repeating NVDA fifty times in a DD post would look like fifty people talking - a single account could fake a crowd.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>set() of extracted tickers per post: each post contributes at most 1 to a ticker's daily count. mention_count therefore = number of DISTINCT posts mentioning the ticker.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Term frequency (count every occurrence).</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>The metric measures breadth of attention, not verbosity. Unit-tested: a post saying '$GME $GME!!' counts exactly once and weighted exactly score^2.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Within-post intensity information is lost.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>build_daily_counts(); test_build_daily_counts_dedupes_and_weights</t>
         </is>
@@ -769,42 +803,47 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Bare matching: original case, 4-5 letters only</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Ticker extraction</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>The extractor originally UPPERCASED text before matching, so every ordinary 'edge'/'loan'/'meme' became a fake ALL-CAPS ticker hit - EDGE and LOAN ranked as top mentioned 'tickers' (18.8k and 17.4k phantom mentions in the 2022 run).</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Cashtags are matched on an uppercased copy ($gme = $GME), but the bare pass runs regex \b[A-Z]{4,5}\b on the ORIGINAL text - only words the author actually typed in caps can match. Cashtag spans are stripped first so $GME doesn't double-count as bare GME. 1-3 letter symbols (A, IT, ALL) can NEVER match bare - cashtag only.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Case-insensitive matching of every universe symbol (maximum recall, terrible precision).</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>'i took out a loan' can never be a $LOAN mention. Precision of the bare pass jumped; the phantom top-tickers vanished.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Genuine lowercase ticker chatter ('gme to the moon') is missed unless cashtagged - precision deliberately chosen over recall.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>src/extract_tickers.py (CASHTAG, WORD_BARE, _strip_cashtags_for_word_pass)</t>
         </is>
@@ -814,42 +853,47 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Word-ticker screening by corpus case ratio</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Word-ticker screening</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Even after the caps fix, real 4-5 letter tickers that are ALSO English words (EDGE, LOAN, RENT, TECH, EARN, CARD, AWAY...) kept polluting the top-20, because people do type them in caps for emphasis. The manual stop list had grown past 200 entries with no end - there are hundreds of word-tickers.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>One pass over a 300k-post sample counts, per candidate symbol, strict-caps occurrences vs any-other-casing occurrences: caps_share = caps / (caps + lower). If the symbol was sighted &gt;= 30 times, caps_share &lt; 0.5 classifies it as a word. The corpus itself votes on what is a word HERE.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Keep growing the hand-maintained stop list forever.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>The measured distribution is strongly bimodal (of 513 symbols with &gt;=30 sightings: 248 below 0.1, 144 above 0.8) - the threshold sits in a real valley. EDGE 0.023, LOAN 0.002, RENT 0.003, SEEM 0.001 vs NVDA 0.931, TSLA 0.926, PLTR 0.937. 423 tickers demoted automatically; verified on Jan-2021: top-20 = GME, AMC, BB, NOK, KOSS... zero word-tickers.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Needs enough sightings; the ratio is era-dependent (measured on the loaded slice - arguably a feature).</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>src/screen_tickers.py; notebook 01 screening section</t>
         </is>
@@ -859,42 +903,47 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>wordfreq as fallback only - corpus wins</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Word-ticker screening</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>~8,700 of the 9,180 candidate symbols appear fewer than 30 times in the sample - no trustworthy ratio - yet each still needs a word/ticker verdict.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>For rare candidates only: zipf_frequency(symbol.lower(), 'en') &gt;= 3.5 classifies it as a common English word. When BOTH signals exist, the corpus ratio decides - the dictionary never overrules observed Reddit usage.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Dictionary-first filtering (wordfreq/NLTK stopwords as the primary screen).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Rare symbols get a sane default with zero corpus cost. Corpus priority rescues real tickers the dictionary calls words: SNAP (zipf 4.21, caps_share 0.56) and AMD (zipf 3.52) survive. Word-tickers score 4.4-5.1 vs real tickers ~2.0-2.6, so 3.5 splits cleanly.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Caps-typed jargon defeats BOTH signals (HODL: zipf 1.73, caps_share 0.62; likewise TLDR) - the manual stop list stays as a third layer.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>classify_ticker() in src/screen_tickers.py</t>
         </is>
@@ -904,42 +953,47 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Demote, don't delete (cashtag_only class)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Word-ticker screening</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Stop-listing LOAN would erase any future ability to detect a genuine retail swarm into the LOAN ticker - a stop list deletes signal forever, silently.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Screened word-tickers get class 'cashtag_only': bare-caps mentions are ignored, but $LOAN still counts. The extractor loads ticker_classification.csv once at import; if the CSV is absent it degrades gracefully to the old behaviour (empty set).</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Binary stop list (delete the symbol entirely).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Prose noise removed with the escape hatch intact: a real spike still surfaces through cashtags. The classification is a reviewable CSV artifact, not code.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Brand-name tickers typed lowercase lose their bare mentions (SOFI 0.34, HOOD 0.25, COIN 0.04) - accepted recall cost, precision-first before Stage 2.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>SCREENED_STOP in src/extract_tickers.py; data/reference/ticker_classification.csv</t>
         </is>
@@ -949,42 +1003,47 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Four-layer stop defence, cheapest first</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Ticker extraction</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>No single filter catches all false-positive modes: made-up symbols, finance jargon (CEO, YOLO, ETF), common English words, and Reddit-specific slang each fail differently.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Ordered layers in the bare pass: (1) Nasdaq-Trader universe membership, (2) STOP_TICKERS jargon list - blocks even cashtags, (3) BARE_PROSE_STOP manual word list, (4) SCREENED_STOP data-driven list. Cashtags are exempt from layers 3-4 by design.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>One monolithic stop list, or ML named-entity recognition.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Each layer is independently inspectable and unit-tested. The corpus layer even catches Reddit-specific usage no dictionary could: ROPE (WSB dark humour, zipf only 4.06) gets demoted by its 0.45 caps_share.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Four lists to reason about; their order matters and must stay documented.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>extract_tickers_from_text()</t>
         </is>
@@ -994,42 +1053,47 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Detect take-offs by first derivative, self-normalised per ticker</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Inflection detection</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>The goal is the MOMENT attention takes off, not who is popular. Absolute levels fail twice: mega-caps are always high (selection bias), and a fixed global threshold can't fit both NVDA (5,000/day) and a small cap (5/day).</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>velocity[t] = smoothed[t] - smoothed[t-1] (3-day rolling mean first). A day is flagged when velocity &gt; mean + K*std computed from THAT ticker's own velocity history (K=2.0); falls symmetric with K below the mean.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Threshold on raw counts, or one global threshold for all tickers.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>The threshold self-normalises: every ticker is judged against its own noise, so a small cap's genuine 5x jump outranks NVDA's daily wobble. Unit-tested: 20 quiet days + a spike flags only the spike.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Differencing doubles level-noise - which forced the smoothing decisions below.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>src/inflection.py; notebook 03; K to be calibrated vs price (Stage 1 step 5)</t>
         </is>
@@ -1039,42 +1103,47 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Smooth on log(1+count) with EWMA</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Inflection detection</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>The velocity plot looked like a saw blade: differencing amplifies noise, a 3-day mean can't kill the weekday/weekend cycle (every Monday looked like a take-off), counts are small integers, and one 3,000-mention viral day flattens everything else on the axis.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Transform to log(1+count), then EWMA with span 14 (exponentially weighted - recent days weigh more), then differentiate. Key property: the derivative of a log is approximately the daily PERCENTAGE growth rate. Threshold K_SMOOTH=2.5 on this smoother signal.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Just widen the simple moving average (reacts too slowly and still arithmetic-scale).</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Velocity becomes a growth rate comparable across big and small tickers; viral days no longer dominate the axis; weekend dips ironed out.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>The smoother the span, the later the flag (1-2 days at span 14) - an explicit, documented knob.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>smooth_inflection() in notebook 03</t>
         </is>
@@ -1084,42 +1153,47 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Peaks/troughs gated by scipy prominence</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Inflection detection</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Naively marking every velocity sign-flip as a 'turning point' flagged dozens of meaningless wiggles per year - annotations became noise themselves.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>scipy.signal.find_peaks on the smoothed line with a prominence floor (0.75 log-units on the EWMA signal; peak_k * std in the classic pass). Prominence = how far a local extreme stands out from its surroundings, not merely that it is one.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Mark every local max/min.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Only bold 'rose here, fell back out' turns get annotated - charts stay readable.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>One more parameter (PEAK_PROMINENCE) to tune per signal scale.</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>notebook 03; src/inflection.py</t>
         </is>
@@ -1129,42 +1203,47 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Two z-scores: rolling AND cross-sectional</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Normalisation</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>'Is this week unusual for THIS ticker?' and 'Who dominates the conversation TODAY?' are different questions - one normalisation can't answer both.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Rolling z: (weekly - 84-day rolling mean) / 84-day rolling std, per ticker, minimum 28 days of history. Cross-sectional z: z-score of log(1+weekly) ACROSS all tickers each day (log so mega-tickers don't define the scale).</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Pick a single normalisation.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Rolling z times a ticker's own take-off regardless of its size; cross-sectional z ranks the day's leaderboard. Used together: 'take-off + climbing the leaderboard' is the strongest read.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Rolling z has a 28-day warm-up - documented advice: start the window ~3 months before the event of interest (e.g. Jan-2021 GME).</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>notebook 02, z-score section</t>
         </is>
@@ -1174,42 +1253,47 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Per-year framing everywhere</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Normalisation</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Archived upvote scores are mature, so 2021's viral posts dominate any all-time chart - both which tickers get picked and the y-axis scale - forever hiding newer years.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>One plot per year; each year ranks its OWN top tickers; inflection thresholds computed within-year so a take-off is judged against that year's noise.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>All-time charts with a global top-N.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Every year competes only with itself; 2024's story is visible next to 2021's.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Cross-year magnitude comparisons need extra care.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>notebooks 02 and 03 (per-year sections)</t>
         </is>
@@ -1219,42 +1303,47 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Volume floor before trend analysis</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Signal construction</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Tickers with a handful of total mentions produce 'trends' that are pure noise - the smoother happily draws a confident line through 7 data points.</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Skip tickers with fewer than MIN_TOTAL=300 total mentions in the window before the smooth-signal inflection pass.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Analyse every ticker that appears.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>No tea-leaf charts; compute is spent on tickers that can actually trend.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>The very earliest whisper stage of a micro-cap is invisible below the floor.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>MIN_TOTAL in notebook 03</t>
         </is>
@@ -1264,42 +1353,47 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Notebook chain with one source of truth</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Pipeline design</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Each notebook had its own TIME WINDOW cells - and they drifted: 02 was found running on 2022 while 01 was set to 2021, so 'the same analysis' silently used different data.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>01 saves the filtered slice to posts_slice.parquet (on by default) plus the screening CSV; 02 and 04 have NO window cells - they read the slice and raise FileNotFoundError('run notebook 01 first') if it is missing; 03/05 already consume 02/04's output files. 02 importlib.reload()s the extractor so a live kernel picks up a re-generated screening CSV.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Independent notebooks with duplicated filter cells (the previous state).</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>The chain 01-&gt;02-&gt;03 / 01-&gt;04-&gt;05 provably shares ONE timeframe; changing the window is a one-cell edit in 01. Verified end-to-end: Jan-2021 slice (666k posts) -&gt; clean top-20 in ~5 s of extraction.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>The slice duplicates ~400 MB on disk for a 1-year window.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>notebooks 01, 02, 04</t>
         </is>
@@ -1309,42 +1403,47 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Staged go/no-go research design</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Research design</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Sentiment scoring (Stage 2) and X/Twitter network analysis (Stage 3) are expensive to build - and pointless if the cheap signal already works, or if no mention signal leads price at all.</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Stage 1 must first show that RAW mention/theme spikes LEAD ETF moves: correlate daily mentions against GLD, MAGS, BTC, SMH returns at shifts of -10..+10 days; the best-correlated lag measures IF and BY HOW MANY DAYS Reddit leads. Only a failure of the raw signal triggers Stage 2.</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Build the full sentiment + network stack up front.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>The cheapest falsifiable test runs first. Spikes are explicitly 'look here', never 'buy' - direction blindness (GME calls vs puts look identical) is acknowledged and deferred to Stage 2.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>If Stage 1 fails, some of its tooling is sunk cost.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>README 'Next steps' (steps 4-6); planned src/price_lag.py + notebook 06</t>
         </is>
@@ -1354,42 +1453,47 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Score-maturity bias handled by design</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Research design</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Archive dumps captured posts long after posting (scores mature); a live-fetched post has score ~0 minutes after creation even if it later goes viral. Weighted counts across the two eras are NOT comparable - a subtle trap that would poison any live back-test.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Ordered mitigations: (a) validate on raw mention_count first - it is immune (one post = 1 either way); (b) for live data, re-poll each post's score after a fixed 24-48h maturation window so both eras are measured at the same age; (c) fallback: compare each day only to its own trailing baseline (z-scores); (d) last resort: soften score^2 to score or log(1+score).</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Ignore it and compare weighted counts directly across eras.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>The trap is documented BEFORE live ingestion exists; the raw-count-first validation order makes Stage 1 immune to it entirely.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Re-polling doubles Reddit API traffic on the paid tier.</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>README 'Historical vs live data' caveat box</t>
         </is>
@@ -1399,42 +1503,47 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Tests pin the DATA, not just the code</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Quality / process</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>A silently bad rebuild (wrong filter, missing dump, re-crawl) would invalidate every downstream result while all code tests still pass green.</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>pytest asserts the dataset itself: exact total rows (7,954,297), exact per-subreddit counts for all 15 subs, date range and strict YYYY-MM-DD format on a sample, duplicate ceiling (&lt;=5). Plus hand-made-example unit tests and an end-to-end run of the real daytrading block (89,512 posts) through the full pipeline, internet-free.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Test only code logic with synthetic fixtures.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>20 checks; any dataset drift fails loudly with the exact expectation printed. The e2e test doubles as a living example of the pipeline.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Row-count assertions must be updated on every INTENTIONAL rebuild.</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>tests/test_pipeline.py</t>
         </is>
@@ -1444,42 +1553,47 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Notebooks treated as fragile JSON</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Quality / process</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>A stale read-modify-write once corrupted two notebook files (folder-sync lag delivered a half-synced file that was then edited and written back).</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Editing rule: parse-first (a successful json.load proves the snapshot is complete) or fully regenerate from known content - never blind string-patching. check_notebooks.py validates/auto-fixes; JSON validity of every notebook is itself a pytest.</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Treat .ipynb as ordinary text files.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Corruption is detected the moment it happens (test fails with line/column) and is recoverable (--fix or regeneration).</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Editing overhead on every notebook change.</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>data_ingestion/scripts/check_notebooks.py; tests group 3</t>
         </is>
@@ -1489,42 +1603,47 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Reproducible, reviewable screening artifact</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Quality / process</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>An unseeded sample would produce a slightly different classification CSV on every run - the extraction layer would be non-deterministic and borderline tickers would flip between runs.</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Sample is seeded (random_state=0, 300k posts); all three thresholds live in ONE module (screen_tickers.py); the output is a committed CSV with the evidence per ticker (caps_count, lower_count, caps_share, zipf, decided_by) - not opaque code.</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Unseeded sampling; thresholds scattered across notebooks.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Re-running notebook 01 reproduces the identical CSV; a threshold change shows up as a reviewable CSV diff; any human can eyeball WHY a ticker was demoted.</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>A different seed would flip a few borderline symbols (documented, not hidden).</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>src/screen_tickers.py; data/reference/ticker_classification.csv</t>
         </is>
@@ -1534,44 +1653,349 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Theme scanning: tokenise once + hash lookups</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>The original theme scanner ran ~20 separate keyword regexes over every post's full text. At ~130-600 posts/sec, a one-year window (2.8M posts) meant HOURS per notebook-04 run - too slow to iterate on.</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>One pass per post: lowercase the text once, tokenise with a single regex ([a-z0-9]+), then look every token up in a prebuilt dict {word -&gt; themes} (O(1) per token, regardless of how many keywords exist). Multi-word phrases ('short squeeze', 'data center') are checked with Python's C-level substring 'in' against the lowered text. Per-post set semantics kept: a post counts at most once per theme.</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Option considered: one combined pre-compiled regex per theme + pandas str.count (vectorised). Hash lookups won: cost is O(tokens in post), not O(number of keywords), so adding keywords is free.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Measured on real data (100k-post benchmark): 12,298 posts/sec -&gt; the full 2.8M-post window takes ~4 minutes instead of ~6 hours (~95x). Stale 'many HOURS' warnings removed from WEEK2.md and notebook 01.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Single-word keywords must match a whole token exactly - plurals/variants need listing explicitly ('chip' AND 'chips'). Phrases are still scanned per post (fast C substring, but linear in phrase count).</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>src/themes.py (themes_in_text, _get_keyword_lookup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Tradeable, ETF-anchored themes</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Signal construction</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Themes like 'options_volatility' or 'earnings' spike in mentions but point at nothing you can buy - a signal with no trade attached is unfalsifiable against prices (JPM's Retail Lens monitors tradeable names/sectors for the same reason).</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Every theme in THEME_KEYWORDS is anchored to one liquid instrument in a new THEME_ETFS map (semiconductors-&gt;SMH, gold_metals-&gt;GLD, uranium_nuclear-&gt;URA, europe_defense-&gt;EUAD, rates_bonds-&gt;TLT...). Vague themes (options chatter, earnings chatter, IPO chatter) were deleted; new tradeable ones added (uranium_nuclear, defense_aerospace, europe_defense). short_squeeze/meme_stocks keep GME as an honest single-stock proxy.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Keep every theme that is interesting to read, tradeable or not.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Each mention/sentiment spike now maps to a back-testable instrument, and the price backtest (notebook 08) can cover every theme, not just the original four ETFs. A pytest enforces that every theme has an anchor.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Some colour is lost (options/earnings chatter can context-flag regimes); europe_defense has thin US-listed coverage (EUAD only) so its inferred-ticker signal is weak - keyword signal carries it.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>src/themes.py (THEME_KEYWORDS, THEME_ETFS, THEME_TICKERS); test_every_theme_has_a_tradeable_anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Sentiment engine: VADER + custom WSB lexicon</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Stage 2 needs direction (bull vs bear), but plain VADER misreads finance ('calls'/'puts' neutral, 'short' generically negative, 'moon'/'tendies' unknown), and finance-tuned transformers (FinBERT/FinTwitBERT) cost GPU-hours plus a heavy dependency - too expensive before the signal has proven ANY value.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>VADER lexicon scorer with ~50 injected WSB/finance terms at hand-set valences (moon +2.5, calls +1.5, puts -1.5, rug -2.5, bagholder -2.5...). Compound score per post in [-1,+1]; selftext truncated at 1,000 chars (sentiment saturates with length). Scored once per slice, cached to parquet, shared by notebooks 06 and 07.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Jump straight to a finance-tuned transformer, or use raw VADER unmodified.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Whole 1-year slice scores in ~20-40 min on CPU, fully offline and explainable (you can point at the exact lexicon entry that moved a score). Verified: bullish slang text +0.81, bearish slang -0.89, neutral text 0.00. Upgrade path: swap the engine behind score_text() if the signal proves out.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Lexicons cannot read sarcasm, loss-porn irony or 'puts printing' - treat levels as noisy and changes-vs-own-baseline as the real read. Token-based: multi-word slang ('diamond hands') only counts via its scoreable parts.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>src/sentiment.py (WSB_LEXICON, score_text, add_sentiment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Headline sentiment metric: net_bullish share, not mean score</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>A daily mean compound score is dragged around by one long, extreme post, and means of small samples (5 posts/day tickers) swing violently - the chart becomes noise.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>net_bullish = (share of posts with compound &gt; +0.05) - (share &lt; -0.05), bounded [-1,+1] ('30 points more bulls than bears'). Noise controls stacked on top: days under MIN_POSTS masked BEFORE smoothing, 7-day rolling means on charts (JPM's published chart is weekly-rolling), and theme-level lines (hundreds of posts/day) preferred over single tickers for regime reads.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Plot the raw daily mean compound score per ticker.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>A bounded, outlier-robust series that reads naturally and matches the JPM-style presentation (5-day arrow strips, monitor tables in notebooks 06/07). Unit-tested: 2 bulls + 1 bear = exactly +1/3.</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Discards intensity (a +0.9 post counts the same as +0.1); avg_sentiment is saved alongside for anyone who wants it.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>src/sentiment.py (_aggregate); notebooks 06/07</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>2-minute runtime budget for sentiment (multithreading + sampling)</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Single-core VADER scoring ran at ~1-3k posts/sec -&gt; 20-40 min for a 1-year slice. Analyst iteration dies at that speed; the requirement was set at &lt;= 2 minutes per notebook run.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Three stacked multipliers in add_sentiment_fast(): (1) MULTIPROCESSING - posts are split into 20k-chunks and scored on every CPU core via joblib (VADER is embarrassingly parallel; each worker builds its own analyzer); (2) truncation tightened 1000 -&gt; 300 chars (~4.5x per core - sentiment saturates in the first few hundred characters); (3) a seeded sample cap (MAX_SCORE_POSTS = 500k, seed 0) as the hard guarantee - net_bullish is a PROPORTION, so 500k sampled posts estimate daily shares within ~1-2 points. Notebooks print a loud banner when sampling and stamp the exact time window into every chart title (also covers the narrower-window fallback).</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Accept the 20-40 min run, or permanently shrink the analysis window.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Measured on a 2-core sandbox: 13,158 posts/sec (vs ~1.2k before) with parallel output verified identical to single-core; on a typical 8-thread machine the 500k cap scores in well under a minute and even the full 2.8M-post year lands near the 2-minute mark. Cache still shared between notebooks 06/07.</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Sampling makes post-volume panels show SCORED posts (proportional, not absolute); results depend on cores available; joblib added as a dependency. Set MAX_SCORE_POSTS=None for exact numbers.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>src/sentiment.py (add_sentiment_fast, _score_batch); notebooks 06/07</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Conviction = mentions x sentiment; sentiment read as CHANGE, not level</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Signal construction</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Mentions are direction-blind (GME calls vs puts identical) and sentiment LEVELS are bullish-biased (retail skews long, bullish slang dominates - measured: nearly every ticker's average net_bullish &gt; 0). Each ingredient alone misleads.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Composite in notebook 08: bull_pressure = n_posts x net_bullish (bullish-minus-bearish POST COUNT: volume and direction in one number), 7d-rolled and z-scored vs each ticker's own history = conviction_z. Divergence flags where the ingredients disagree (attention z &gt; 1 while 5d sentiment change &lt; -0.1 = crowded-top risk; both rising = confirmed swarm). Momentum maps' y-axis switched from sentiment LEVEL to CHANGE (last 5d minus own window average), cancelling the per-name bullish bias. Weekly heatmaps + monthly snail trails unroll the snapshot over time.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Use either signal alone, or plot absolute sentiment levels.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>One bounded composite per ticker/day (daily_ticker_conviction.parquet) ready for the price backtest (notebook 09); the change-based map makes bearish shifts visible despite the bullish floor; masking floor auto-scales with the sentiment sample fraction (fixed the 'gaps in the chart' artifact).</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>z-scoring removes each name's constant bias but market-wide mood swings still move all names together (information, not noise); divergence flags are descriptive until backtested.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>notebooks/08_retail_conviction.ipynb; notebooks 06/07 maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard reads only derived parquets, never raw data</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Pipeline design</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>A monitoring UI that recomputes from the 1.15 GB posts parquet would be slow, and one that fabricates demo data would be worse than nothing.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Streamlit app (dashboard/app.py) reads ONLY the notebooks' saved outputs (daily_ticker_counts, by_source, ticker/theme sentiment parquets). Sidebar timeframe picker (presets + custom range) re-filters every panel - KPIs, top mentions, top velocity-change (z of day-over-day 7d-rolling mentions), JPM-style market/theme sentiment lines, interactive momentum map, Reddit-vs-X split. File mtime is part of the cache key, so re-running a notebook refreshes the dashboard automatically. Panels whose input file is missing show 'run notebook X first' - no synthetic placeholders anywhere.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Recompute from raw posts in the app, or mock data for missing panels.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Instant timeframe changes on cached frames; a clean contract: notebooks produce, dashboard displays; the same app will show live data the moment live ingestion refreshes the parquets.</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard is only as fresh as the last notebook run; velocity/momentum stats are window-relative, so changing the timeframe changes the baselines (by design).</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>dashboard/app.py; streamlit run dashboard/app.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ready for backtest, pre-financial data but all working so far with trading signals (not tested). trading logic needs to be tweaked
</commit_message>
<xml_diff>
--- a/design_decisions.xlsx
+++ b/design_decisions.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1996,6 +1996,206 @@
       <c r="J30" s="2" t="inlineStr">
         <is>
           <t>dashboard/app.py; streamlit run dashboard/app.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>REMOVED the score-squared upvote weighting (look-ahead leak)</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Signal construction</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Archived Reddit dumps store each post's FINAL score - upvotes collected days or weeks AFTER posting. weighted_count therefore let day-t signals 'know' which posts would go viral: a look-ahead leak that silently inflates any backtest built on it. Discovered while designing the trade backtest; overrides decision #4.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>build_mentions.py now returns date/ticker/mention_count only; notebook 02's weighted graphs deleted; the theme columns keyword_weighted/inferred_weighted are kept for notebook compatibility but hard-set to 0 (deprecated); a pytest asserts the weighted column stays gone. Notebooks 03/05 already fall back to mention_count when the column is missing.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Keep the weighted signal 'for description only' and trust everyone to remember not to backtest on it.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>The backtest path is leak-free by construction, not by discipline. If weighting ever returns it must use scores AS OF the mention day (live 24-48h re-poll pipeline).</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Loses the viral-vs-noise distinction until a point-in-time score source exists; old saved parquets with weighted columns are stale.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>src/build_mentions.py, src/themes.py, notebook 02, tests; README 'Why there is NO upvote-weighted signal'</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Survivorship fix: hand-curated DELISTED_TICKERS supplement</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Data engineering</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>The ticker universe is downloaded from today's Nasdaq Trader files, so delisted names (BBBY, SPRT, WISH...) vanish - and their historical mentions silently stop counting. The casualties are exactly the names retail piled into before they died, so the omission flatters any backtest (survivorship bias).</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>A curated frozenset of 14 known dead retail favourites is unioned into the universe at load time (bankrupt/acquired/delisted meme names, each dated in a comment). Extend the set whenever a name known to be loud on Reddit fails to appear in notebook 02's tables.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Ignore it (bias), or build a full point-in-time universe from archived nasdaqlisted.txt snapshots / Bloomberg/CRSP exports.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>The famous casualties count again with a one-line change per name; pytest validates every supplement symbol. The point-in-time universe remains the proper long-term fix (logged in the README live-data checklist) - a hand list can never be complete.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Manual and inherently incomplete; single-ticker backtests also need delisted PRICE data (Bloomberg has it) - theme-ETF backtests are immune to both problems.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>src/ticker_universe.py (DELISTED_TICKERS); test_delisted_supplement_fixes_survivorship</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Signal generation separated from price evaluation (notebook 09)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Pipeline design</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Trading decisions and their evaluation kept blurring together in discussion: 'what would we buy' depends only on OUR data; 'did it work' needs price data the repo doesn't have yet. Mixing them in one notebook invites accidentally tuning entries against the prices they are judged on.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Notebook 09 produces ONLY the entry log (trade_signals.parquet: signal date, next-day buy date, theme, anchor ETF, S1/S2 trigger, conviction score 0-5 with the checks that fired) using TRAILING 84d baselines exclusively - never whole-window statistics - so the identical code runs on live data later. Entries fire on threshold CROSSINGS (yesterday &lt;= K, today &gt; K), not levels, so one surge = one entry, not a buy every day above K. The price backtest lives separately in notebook 10 and consumes 09's log.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>One combined notebook that generates signals and scores them against prices in the same place.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Verified on constructed data: a single surge produces exactly one crossing, nothing fires during the 28-day warm-up, score assembly matches the WEEK2 stacking rules. When live ingestion lands, 09 IS the daily signal run (plus snapshot discipline).</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Without prices the signals are unvalidated paper entries; the score is logged, not used for sizing, until notebook 10 shows high scores actually outperform.</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>notebooks/09_trading_signals.ipynb; data/processed/trade_signals.parquet</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Conjunctive entry gate: momentum AND sentiment must agree (fewer trades, more conviction)</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Signal construction</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>A momentum-only rule trades every attention spike, including panic spikes and pump-and-dumps; a sentiment-only rule trades noise. Trading each alone produces many low-quality entries.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Notebook 09 v2: a BUY needs ALL of (1) a momentum CROSSING (attention z or conviction z crosses above +K), (2) sentiment agreement (5d change of net-bullish share &gt; 0), and (3) conviction score &gt;= MIN_SCORE (4 of 5 checks). SELL is the mirror (conviction crosses below -K or crowded-top divergence activates, 5d sentiment change &lt; 0, score &gt;= 3 - lower bar because the retail bullish floor makes bearish checks structurally harder). Every trade carries a plain-language reason string with the actual numbers behind each conviction point.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Trade every threshold crossing and let the backtest sort it out.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Verified on constructed cases: momentum cross with disagreeing sentiment produces NO trade; the sell path fires at the bearish cross; sub-threshold scores are filtered. Trade count drops sharply by construction - each surviving entry is explainable line by line.</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>A conjunctive gate can miss moves where sentiment lags attention by more than 5 days; MIN_SCORE adds a parameter that notebook 10 must sanity-check (does score 5 beat score 4?).</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>notebooks/09_trading_signals.ipynb (v2); trade_signals.parquet gains action + reason columns</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data ingestion kind of works but dashboard / reddit live ingestion does not work yet
</commit_message>
<xml_diff>
--- a/design_decisions.xlsx
+++ b/design_decisions.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2196,6 +2196,256 @@
       <c r="J34" s="2" t="inlineStr">
         <is>
           <t>notebooks/09_trading_signals.ipynb (v2); trade_signals.parquet gains action + reason columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Sentiment engines: VADER for backfill, FinTwitBERT for live (calibrated on StockTwits labels)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>fintwit-bot (studied as reference project) uses FinTwitBERT-sentiment - a BERT fine-tuned on finance tweets, genuinely more accurate per post than our VADER lexicon. Should we switch?</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Volume decides, not accuracy alone: BERT on CPU is ~50-200 posts/sec -&gt; DAYS for the 10.8M-post backfill (VADER+parallel = minutes), and our signals aggregate hundreds of posts where lexicon noise averages out. LIVE volume is thousands/day -&gt; FinTwitBERT costs ~1 min/day there. Plan: keep VADER for history; before go-live, score a month of StockTwits messages with BOTH engines and compare against the authors' OWN bullish/bearish labels (ground truth); adopt FinTwitBERT live only if it wins. Engine swap is one function (score_text) - downstream untouched.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Switch everything to FinTwitBERT now, or never upgrade.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Backfill stays fast and reproducible; the live upgrade is evidence-gated instead of vibes-gated; calibration data is free (StockTwits).</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Two engines = two sentiment scales; never mix scores across the switch without re-baselining (z-scores handle this).</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>data_ingestion/LIVE_INGESTION.md; src/sentiment.py (score_text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>StockTwits adopted as third source (self-labelled sentiment = free ground truth)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Data engineering</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>No key needed, finance-native, and unique among our sources: users label their own posts Bullish/Bearish - the only ground truth available for validating ANY sentiment engine on finance-social text.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>fetch_stocktwits.py polls the public symbol streams (~40 symbols = theme ETF anchors + retail favourites) hourly, appends RAW jsonl.zst (labels preserved there); src/stocktwits_data.py normalises to the 9-column schema (id prefix st_, subreddit/source = stocktwits). Rate care: ~200 req/h unauth cap, fetcher stops on 429.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Ignore StockTwits, or scrape it without rate care.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>A live social source that works TODAY with zero credentials, plus the calibration dataset for decision #34. Verified: normaliser schema/dedup/drop rules + label extraction all green.</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Only ~30 messages per symbol per poll (shallow history - it accumulates going forward, no backfill); labels are voluntary (many posts unlabelled).</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>data_ingestion/scripts/fetch_stocktwits.py; src/stocktwits_data.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Output surface: the dashboard ONLY (Discord alerting built, then removed same day)</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Pipeline design</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>fintwit-bot's UI is a Discord bot. We briefly adopted a webhook-alert version, then decided a single output surface beats scattered pings: monitoring, updates AND trade decisions should live in one place.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>src/alerts.py was deleted; the Streamlit dashboard gained a SIGNALS panel that reads notebook 09's trade_signals*.parquet and shows every BUY/SELL with its date, instrument, conviction score and full reason string, filtered by the dashboard's timeframe picker like every other panel. Discord-as-ingestion remains rejected (consent/ToS).</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Keep webhook alerts alongside the dashboard, or a full Discord bot.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>One place to look; signals sit next to the mention/sentiment context that produced them; no secrets to manage (webhook URL removed from example.env).</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>No push notifications - you must open the dashboard; if push is ever wanted again, the webhook pattern is in git history.</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>dashboard/app.py (signals panel); example.env; data_ingestion/LIVE_INGESTION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>X live pipeline built ARMED-BUT-OFF (activates when a paid API key appears)</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Pipeline design</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Live X data needs the paid official API; the decision to pay is pending. Waiting to BUILD until after paying would couple a spending decision to an engineering delay - and risk a rushed integration later.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>fetch_x_live.py is fully built against the official v2 recent-search endpoint: cashtag queries from THEME_ETFS (chunked ~12 per query, lang:en, no retweets), --max-tweets budget seat belt, instant stop on 429, appends to data/raw/X Data/x_api_live.csv.zst with cross-run id dedup. That file is a REGISTERED dataset (normalise_x_api in src/x_data.py) sharing the x_ id prefix with the historical dumps, so add_x_data.py merges it with zero changes and overlaps dedupe automatically. Without X_BEARER_TOKEN in .env the script prints 'armed but off' and exits cleanly - the day the user pays, pasting one token lights up the whole leg.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Build the integration only after paying, or rely on the ToS-risky curl-replay trick.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Verified: normaliser (prefix/date/likes/dedup/bad-date), cross-run append dedup round trip, registry skip in fetch_x_data (repo=None), and the no-token exit path. Total activation cost when paying: paste one line into .env.</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Untestable against the real API until paid (endpoint/params could drift - check developer.x.com docs on activation day); quota maths must be redone against the tier actually purchased.</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>data_ingestion/scripts/fetch_x_live.py; src/x_data.py (normalise_x_api, x_api_live registry entry); example.env; LIVE_INGESTION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Daily orchestration executes the NOTEBOOKS in place (nbconvert), not a parallel script pipeline</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Pipeline design</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Live mode needs an unattended daily run (fetch -&gt; merge -&gt; compute -&gt; snapshot). The obvious approach - reimplementing the notebook logic in a standalone script - creates a second copy of the pipeline that WILL drift from the notebooks the user actually reads and edits.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>run_daily.py executes the existing notebooks with jupyter nbconvert --execute --inplace, in chain order (01-&gt;02-&gt;06-&gt;07-&gt;09), after running the enabled fetchers and a conditional X-block merge (only when the live raw file is newer than the parquet). Signals are snapshotted daily to signal_snapshots/&lt;date&gt;_*.parquet and never overwritten (the point-in-time record for backtest-to-live comparison). Prerequisite: notebook 01's END_DATE=None so the window self-extends. Trigger: Windows Task Scheduler daily, or the dashboard sidebar button (same script, then cache-clear + reload).</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>A separate headless pipeline script duplicating the notebook logic, or papermill with parameter injection.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>One source of truth: whatever the notebooks say IS what ran; after each run the notebooks contain fresh outputs for inspection. Dry-run verified end-to-end (correct order, conditional merge, snapshot naming, reddit placeholder skip). Caches make no-new-data runs cheap.</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Notebook execution is slower than a bare script and a broken notebook cell halts the chain (by design - fail loudly); Windows file locks require closing Jupyter before merge days.</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>run_daily.py; dashboard sidebar button; LIVE_INGESTION.md 'Automation'</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
live scripts (not updated but using fable)
</commit_message>
<xml_diff>
--- a/design_decisions.xlsx
+++ b/design_decisions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexd\Desktop\GIC\RetailFlow1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C70264-3465-4402-BD59-DB538D622B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F78ED6-DCCC-422B-B525-E282F857C890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2880" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="387">
   <si>
     <t>#</t>
   </si>
@@ -1192,6 +1192,23 @@
     <t>1. Fix: For any candidate symbol seen 30+ times, compute caps_share = (times written in caps) / (times written in caps + times written in any other casing). If caps_share &lt; 0.5, call it a word, not a ticker.
 Why it works: People are consistent without realizing it. If EDGE is 97.7% lowercase in normal sentences, that's a word being used as a word. If NVDA is 93% caps, that's a ticker being used as a ticker. The data splits cleanly into two piles (248 symbols clearly words, 144 clearly tickers) instead of one blurry mess — so the threshold isn't a guess, it's sitting in a real gap in the distribution. 2. Problem: ~8,700 of 9,180 candidate symbols don't show up often enough (&lt; 30 times) to trust the case-ratio math from entry 7. But you still need a verdict on each one.
 Fix: For these rare symbols, use an outside dictionary tool (wordfreq) that scores how common a word is in everyday English (a "zipf" score). Above 3.5 → treat as a common word. But — if a symbol has both enough sightings for the corpus ratio and a dictionary score, the corpus ratio always wins; the dictionary is only used when you have nothing else. Fix: Instead of deleting these symbols, give them a status: cashtag_only. Bare mentions of "LOAN" in text are ignored (too noisy), but $LOAN (with the cashtag) still counts as a real signal.</t>
+  </si>
+  <si>
+    <t>Words like rug, bag, moon, mean nothing to finbert so we need a specific social media traiend NLP</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Why better than embedding: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Identifies ALL CAPS, or !!! Also, it is more explainable as we can see each word score sentiment (like a sum) so vs embedded we get the same result everytime and we can tweak it. Also, we can add new words that come about easy, e.g. how would AI know what tendies or POG is? Embedding trained on wikipedia? so how does it know WSB slang</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1328,7 +1345,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1368,6 +1385,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2973,7 +2996,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13C7ABEF-E5FD-48E1-BB30-4518113B78D4}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
@@ -3270,157 +3293,185 @@
       <c r="I13" s="11"/>
       <c r="J13" s="11"/>
     </row>
-    <row r="14" spans="1:10" ht="127.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+    <row r="14" spans="1:10" ht="135" x14ac:dyDescent="0.25">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="17" t="s">
+        <v>385</v>
+      </c>
+      <c r="G14" s="16"/>
+      <c r="H14" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+    </row>
+    <row r="15" spans="1:10" ht="127.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
         <v>24</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="102" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
-        <v>25</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>185</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>25</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D17" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I17" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="153" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+    <row r="18" spans="1:10" ht="153" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
         <v>34</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C18" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I18" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
         <v>381</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-    </row>
-    <row r="19" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+    </row>
+    <row r="21" spans="1:10" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
         <v>35</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H21" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I21" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>270</v>
       </c>
     </row>
@@ -3429,7 +3480,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A20:J20"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:J2"/>
   </mergeCells>

</xml_diff>